<commit_message>
updates - drop rearrangement, sample control plots near treatments, sample complete burning transects
</commit_message>
<xml_diff>
--- a/documents/Site and Predictor Decisions.xlsx
+++ b/documents/Site and Predictor Decisions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/48d5e44bbfd1f651/Documents/fuels-analysis/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_F25DC773A252ABDACC104889019870845BDE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA17AFD0-E136-483A-9D35-A8EE2DEE2E4C}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_F25DC773A252ABDACC104889019870845BDE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B1A69ED-BAC6-44C7-91A5-6B6EE49CB5B5}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fires Removed" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="76">
   <si>
     <t>Fire Name</t>
   </si>
@@ -148,9 +148,6 @@
     <t>HLI</t>
   </si>
   <si>
-    <t>DailyAreaBurned</t>
-  </si>
-  <si>
     <t>Extreme</t>
   </si>
   <si>
@@ -215,6 +212,48 @@
   </si>
   <si>
     <t>OK either way, can run model with and without</t>
+  </si>
+  <si>
+    <t>Removing because the anomalies, especially temperature, has a very backwards PDP. Elevation and Daily Area Burned should capture climate sufficiently</t>
+  </si>
+  <si>
+    <t>Removing because it is the total count for the plot, so it does not really capture re-entry like I had been thinking. Very low importance as well.</t>
+  </si>
+  <si>
+    <t>Change to weighted treatment age</t>
+  </si>
+  <si>
+    <t>Multicollinearity with Prop_Treated, choosing overall Prop_Treated</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Hectares</t>
+  </si>
+  <si>
+    <t>Daily_Area</t>
+  </si>
+  <si>
+    <t>Daily_Spread</t>
+  </si>
+  <si>
+    <t>Meters</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Daily unidirectional spread (Harris)</t>
+  </si>
+  <si>
+    <t>(Harris)</t>
+  </si>
+  <si>
+    <t>(Balik)</t>
+  </si>
+  <si>
+    <t>This splits a lot of the info from prop_hardwood when compared to prop_aspen. High aspen plots get split between this variable and prop_hardwood. Deciding still to drop though due to multicollinearity. Deciding not to use SAF groups because of multicollinearity with elevation</t>
   </si>
 </sst>
 </file>
@@ -769,7 +808,7 @@
         <v>23</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -779,165 +818,217 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3BD25C5-1441-4BE5-89F3-EF8D2BD00523}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="20.453125" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" customWidth="1"/>
+    <col min="4" max="4" width="29.36328125" customWidth="1"/>
+    <col min="5" max="5" width="17.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
         <v>40</v>
       </c>
-      <c r="C6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+      <c r="D8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
         <v>41</v>
       </c>
-      <c r="C7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
+      <c r="E9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
+      <c r="E10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
+      <c r="E12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
+      <c r="E13" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B13" t="s">
+      <c r="E14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B14" t="s">
+      <c r="E15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B15" t="s">
+      <c r="E16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B16" t="s">
+      <c r="E17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B17" t="s">
+      <c r="E18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="C18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B19" t="s">
+      <c r="E20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
         <v>53</v>
       </c>
-      <c r="C19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
+      <c r="E21" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
         <v>54</v>
       </c>
-      <c r="C20" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
+      <c r="E22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
         <v>55</v>
       </c>
-      <c r="C21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B23" t="s">
+      <c r="E24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
         <v>57</v>
       </c>
-      <c r="C23" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B25" t="s">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B26" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>